<commit_message>
Update chart images and report data from latest pipeline run
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/classification_feedback.xlsx
+++ b/classification_feedback.xlsx
@@ -700,7 +700,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Generated: 2026-02-11 16:48</t>
+          <t>Generated: 2026-02-27 12:35</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -3070,7 +3070,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3754,7 +3754,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3925,7 +3925,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>82%</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>89%</t>
+          <t>84%</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -4609,7 +4609,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -4780,7 +4780,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -5635,7 +5635,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -5749,7 +5749,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -5806,7 +5806,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -5863,7 +5863,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -6205,7 +6205,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>99%</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -6661,7 +6661,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -6775,7 +6775,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -6889,7 +6889,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -7003,7 +7003,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -7060,7 +7060,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -7117,7 +7117,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -7231,7 +7231,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -7288,7 +7288,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -7459,7 +7459,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -7516,7 +7516,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -7573,7 +7573,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -7630,7 +7630,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -7915,7 +7915,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -7972,7 +7972,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -8029,7 +8029,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -8143,7 +8143,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -8257,7 +8257,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -8485,7 +8485,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>89%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>84%</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -8713,7 +8713,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -8770,7 +8770,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -8884,7 +8884,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -8941,7 +8941,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
@@ -9112,7 +9112,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
@@ -9169,7 +9169,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -9226,7 +9226,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
@@ -9283,7 +9283,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
@@ -9340,7 +9340,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
@@ -9397,7 +9397,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -9454,7 +9454,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -9568,7 +9568,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
@@ -9625,7 +9625,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
@@ -9682,7 +9682,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -9739,7 +9739,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -9796,7 +9796,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -9853,7 +9853,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -10024,7 +10024,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -10138,7 +10138,7 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -10252,7 +10252,7 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -10309,7 +10309,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -10366,7 +10366,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -10423,7 +10423,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -10480,7 +10480,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -10537,7 +10537,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -10651,7 +10651,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
@@ -10765,7 +10765,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>84%</t>
+          <t>78%</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -10879,7 +10879,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
@@ -10936,7 +10936,7 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -10993,7 +10993,7 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -11164,7 +11164,7 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -11221,7 +11221,7 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -11278,7 +11278,7 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
@@ -11335,7 +11335,7 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>89%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
@@ -11449,7 +11449,7 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -11506,7 +11506,7 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -11563,7 +11563,7 @@
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -11620,7 +11620,7 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -11677,7 +11677,7 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -11734,7 +11734,7 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -11791,7 +11791,7 @@
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -11848,7 +11848,7 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -11905,7 +11905,7 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -11962,7 +11962,7 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -12019,7 +12019,7 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -12076,7 +12076,7 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -12133,7 +12133,7 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -12190,7 +12190,7 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -12247,7 +12247,7 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -12304,7 +12304,7 @@
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -12361,7 +12361,7 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -12418,7 +12418,7 @@
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -12475,7 +12475,7 @@
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -12532,7 +12532,7 @@
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>84%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
@@ -12760,7 +12760,7 @@
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -12817,7 +12817,7 @@
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
@@ -12874,7 +12874,7 @@
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
@@ -12931,7 +12931,7 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>84%</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -13159,7 +13159,7 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -13216,7 +13216,7 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
@@ -13330,7 +13330,7 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -13387,7 +13387,7 @@
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
@@ -13444,7 +13444,7 @@
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
@@ -13501,7 +13501,7 @@
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
@@ -13558,7 +13558,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
@@ -13615,7 +13615,7 @@
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
@@ -13786,7 +13786,7 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>89%</t>
+          <t>83%</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
@@ -13900,7 +13900,7 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J231" t="inlineStr">
@@ -13957,7 +13957,7 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
@@ -14014,7 +14014,7 @@
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
@@ -14071,7 +14071,7 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J234" t="inlineStr">
@@ -14128,7 +14128,7 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
@@ -14185,7 +14185,7 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
@@ -14242,7 +14242,7 @@
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
@@ -14299,7 +14299,7 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
@@ -14356,7 +14356,7 @@
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
@@ -14413,7 +14413,7 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
@@ -14527,7 +14527,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
@@ -14584,7 +14584,7 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
@@ -14641,7 +14641,7 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
@@ -14698,7 +14698,7 @@
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
@@ -14755,7 +14755,7 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
@@ -14983,7 +14983,7 @@
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
@@ -15154,7 +15154,7 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
@@ -15211,7 +15211,7 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
@@ -15268,7 +15268,7 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
@@ -15325,7 +15325,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
@@ -15382,7 +15382,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -15439,7 +15439,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -15496,7 +15496,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -15553,7 +15553,7 @@
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
@@ -15610,7 +15610,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -15667,7 +15667,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -15724,7 +15724,7 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
@@ -15781,7 +15781,7 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
@@ -15895,7 +15895,7 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
@@ -16066,7 +16066,7 @@
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
@@ -16123,7 +16123,7 @@
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
@@ -16180,7 +16180,7 @@
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
@@ -16237,7 +16237,7 @@
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
@@ -16294,7 +16294,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
@@ -16351,7 +16351,7 @@
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
@@ -16408,7 +16408,7 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
@@ -16465,7 +16465,7 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
@@ -16579,7 +16579,7 @@
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
@@ -16693,7 +16693,7 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>83%</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
@@ -16921,7 +16921,7 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
@@ -17092,7 +17092,7 @@
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
@@ -17149,7 +17149,7 @@
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J288" t="inlineStr">
@@ -17206,7 +17206,7 @@
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J289" t="inlineStr">
@@ -17263,7 +17263,7 @@
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="J290" t="inlineStr">
@@ -17320,7 +17320,7 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J291" t="inlineStr">
@@ -17377,7 +17377,7 @@
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="J292" t="inlineStr">
@@ -17434,7 +17434,7 @@
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
@@ -17491,7 +17491,7 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="J294" t="inlineStr">
@@ -17605,7 +17605,7 @@
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
@@ -17662,7 +17662,7 @@
       </c>
       <c r="I297" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
@@ -17719,7 +17719,7 @@
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
@@ -17776,7 +17776,7 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
@@ -17833,7 +17833,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
@@ -17890,7 +17890,7 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
@@ -17947,7 +17947,7 @@
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
@@ -18004,7 +18004,7 @@
       </c>
       <c r="I303" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>79%</t>
         </is>
       </c>
       <c r="J303" t="inlineStr">
@@ -18061,7 +18061,7 @@
       </c>
       <c r="I304" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J304" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="J305" t="inlineStr">
@@ -18175,7 +18175,7 @@
       </c>
       <c r="I306" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J306" t="inlineStr">
@@ -18232,7 +18232,7 @@
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J307" t="inlineStr">
@@ -18289,7 +18289,7 @@
       </c>
       <c r="I308" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J308" t="inlineStr">
@@ -18346,7 +18346,7 @@
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J309" t="inlineStr">
@@ -18403,7 +18403,7 @@
       </c>
       <c r="I310" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>83%</t>
         </is>
       </c>
       <c r="J310" t="inlineStr">
@@ -18460,7 +18460,7 @@
       </c>
       <c r="I311" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J311" t="inlineStr">
@@ -18517,7 +18517,7 @@
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="J312" t="inlineStr">
@@ -18574,7 +18574,7 @@
       </c>
       <c r="I313" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="J313" t="inlineStr">
@@ -18631,7 +18631,7 @@
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="J314" t="inlineStr">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J315" t="inlineStr">
@@ -18745,7 +18745,7 @@
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J316" t="inlineStr">
@@ -18916,7 +18916,7 @@
       </c>
       <c r="I319" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J319" t="inlineStr">
@@ -19030,7 +19030,7 @@
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J321" t="inlineStr">
@@ -19087,7 +19087,7 @@
       </c>
       <c r="I322" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J322" t="inlineStr">
@@ -19144,7 +19144,7 @@
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J323" t="inlineStr">
@@ -19201,7 +19201,7 @@
       </c>
       <c r="I324" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J324" t="inlineStr">
@@ -19258,7 +19258,7 @@
       </c>
       <c r="I325" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="J325" t="inlineStr">
@@ -19372,7 +19372,7 @@
       </c>
       <c r="I327" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="J327" t="inlineStr">
@@ -19429,7 +19429,7 @@
       </c>
       <c r="I328" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J328" t="inlineStr">
@@ -19543,7 +19543,7 @@
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J330" t="inlineStr">
@@ -19600,7 +19600,7 @@
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J331" t="inlineStr">
@@ -19657,7 +19657,7 @@
       </c>
       <c r="I332" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J332" t="inlineStr">
@@ -19709,12 +19709,12 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>🟡 Moderate (30-50%)</t>
+          <t>🟢 Low (&lt;30%)</t>
         </is>
       </c>
       <c r="I333" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="J333" t="inlineStr">
@@ -19771,7 +19771,7 @@
       </c>
       <c r="I334" t="inlineStr">
         <is>
-          <t>72%</t>
+          <t>78%</t>
         </is>
       </c>
       <c r="J334" t="inlineStr">
@@ -19823,12 +19823,12 @@
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>🟠 Elevated (50-70%)</t>
+          <t>🔴 High Risk (&gt;70%)</t>
         </is>
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="J335" t="inlineStr">
@@ -19885,7 +19885,7 @@
       </c>
       <c r="I336" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J336" t="inlineStr">
@@ -19942,7 +19942,7 @@
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J337" t="inlineStr">
@@ -19999,7 +19999,7 @@
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J338" t="inlineStr">
@@ -20056,7 +20056,7 @@
       </c>
       <c r="I339" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J339" t="inlineStr">
@@ -20113,7 +20113,7 @@
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="J340" t="inlineStr">
@@ -20170,7 +20170,7 @@
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J341" t="inlineStr">
@@ -20227,7 +20227,7 @@
       </c>
       <c r="I342" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J342" t="inlineStr">
@@ -20284,7 +20284,7 @@
       </c>
       <c r="I343" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J343" t="inlineStr">
@@ -20341,7 +20341,7 @@
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="J344" t="inlineStr">
@@ -20398,7 +20398,7 @@
       </c>
       <c r="I345" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="J345" t="inlineStr">
@@ -20455,7 +20455,7 @@
       </c>
       <c r="I346" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J346" t="inlineStr">
@@ -20512,7 +20512,7 @@
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J347" t="inlineStr">
@@ -20564,12 +20564,12 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>🟠 Elevated (50-70%)</t>
+          <t>🔴 High Risk (&gt;70%)</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="J348" t="inlineStr">
@@ -20626,7 +20626,7 @@
       </c>
       <c r="I349" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="J349" t="inlineStr">
@@ -20683,7 +20683,7 @@
       </c>
       <c r="I350" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J350" t="inlineStr">
@@ -20740,7 +20740,7 @@
       </c>
       <c r="I351" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="J351" t="inlineStr">
@@ -20797,7 +20797,7 @@
       </c>
       <c r="I352" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J352" t="inlineStr">
@@ -20854,7 +20854,7 @@
       </c>
       <c r="I353" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="J353" t="inlineStr">
@@ -20906,12 +20906,12 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>🟡 Moderate (30-50%)</t>
+          <t>🟢 Low (&lt;30%)</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="J354" t="inlineStr">
@@ -20968,7 +20968,7 @@
       </c>
       <c r="I355" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="J355" t="inlineStr">
@@ -21082,7 +21082,7 @@
       </c>
       <c r="I357" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="J357" t="inlineStr">
@@ -21196,7 +21196,7 @@
       </c>
       <c r="I359" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="J359" t="inlineStr">
@@ -21310,7 +21310,7 @@
       </c>
       <c r="I361" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="J361" t="inlineStr">
@@ -21367,7 +21367,7 @@
       </c>
       <c r="I362" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J362" t="inlineStr">
@@ -21424,7 +21424,7 @@
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="J363" t="inlineStr">
@@ -21481,7 +21481,7 @@
       </c>
       <c r="I364" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J364" t="inlineStr">
@@ -21538,7 +21538,7 @@
       </c>
       <c r="I365" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J365" t="inlineStr">
@@ -21595,7 +21595,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J366" t="inlineStr">
@@ -21652,7 +21652,7 @@
       </c>
       <c r="I367" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J367" t="inlineStr">
@@ -21709,7 +21709,7 @@
       </c>
       <c r="I368" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>80%</t>
         </is>
       </c>
       <c r="J368" t="inlineStr">
@@ -21766,7 +21766,7 @@
       </c>
       <c r="I369" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J369" t="inlineStr">
@@ -21823,7 +21823,7 @@
       </c>
       <c r="I370" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J370" t="inlineStr">
@@ -21880,7 +21880,7 @@
       </c>
       <c r="I371" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J371" t="inlineStr">
@@ -21937,7 +21937,7 @@
       </c>
       <c r="I372" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J372" t="inlineStr">
@@ -22051,7 +22051,7 @@
       </c>
       <c r="I374" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="J374" t="inlineStr">
@@ -22108,7 +22108,7 @@
       </c>
       <c r="I375" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J375" t="inlineStr">
@@ -22165,7 +22165,7 @@
       </c>
       <c r="I376" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J376" t="inlineStr">
@@ -22222,7 +22222,7 @@
       </c>
       <c r="I377" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="J377" t="inlineStr">
@@ -22279,7 +22279,7 @@
       </c>
       <c r="I378" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="J378" t="inlineStr">
@@ -22336,7 +22336,7 @@
       </c>
       <c r="I379" t="inlineStr">
         <is>
-          <t>78%</t>
+          <t>79%</t>
         </is>
       </c>
       <c r="J379" t="inlineStr">
@@ -22393,7 +22393,7 @@
       </c>
       <c r="I380" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J380" t="inlineStr">
@@ -22450,7 +22450,7 @@
       </c>
       <c r="I381" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J381" t="inlineStr">
@@ -22507,7 +22507,7 @@
       </c>
       <c r="I382" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J382" t="inlineStr">
@@ -22564,7 +22564,7 @@
       </c>
       <c r="I383" t="inlineStr">
         <is>
-          <t>89%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J383" t="inlineStr">
@@ -22621,7 +22621,7 @@
       </c>
       <c r="I384" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>79%</t>
         </is>
       </c>
       <c r="J384" t="inlineStr">
@@ -22678,7 +22678,7 @@
       </c>
       <c r="I385" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J385" t="inlineStr">
@@ -22792,7 +22792,7 @@
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="J387" t="inlineStr">
@@ -22849,7 +22849,7 @@
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J388" t="inlineStr">
@@ -22906,7 +22906,7 @@
       </c>
       <c r="I389" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J389" t="inlineStr">
@@ -22963,7 +22963,7 @@
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="J390" t="inlineStr">
@@ -23020,7 +23020,7 @@
       </c>
       <c r="I391" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>88%</t>
         </is>
       </c>
       <c r="J391" t="inlineStr">
@@ -23077,7 +23077,7 @@
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J392" t="inlineStr">
@@ -23134,7 +23134,7 @@
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="J393" t="inlineStr">
@@ -23191,7 +23191,7 @@
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J394" t="inlineStr">
@@ -23248,7 +23248,7 @@
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t>96%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="J395" t="inlineStr">
@@ -23305,7 +23305,7 @@
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="J396" t="inlineStr">
@@ -23362,7 +23362,7 @@
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="J397" t="inlineStr">

</xml_diff>